<commit_message>
Changes for final review was done
</commit_message>
<xml_diff>
--- a/Marhaba v4/public/pivot-template.xlsx
+++ b/Marhaba v4/public/pivot-template.xlsx
@@ -35257,7 +35257,7 @@
     <pageField fld="3" hier="-1"/>
   </pageFields>
   <dataFields count="1">
-    <dataField fld="14" subtotal="count"/>
+    <dataField fld="14" subtotal="count" numFmtId="1"/>
   </dataFields>
   <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
 </pivotTableDefinition>
@@ -35396,7 +35396,7 @@
     <pageField fld="3" hier="-1"/>
   </pageFields>
   <dataFields count="1">
-    <dataField fld="12" subtotal="average"/>
+    <dataField fld="12" subtotal="average" numFmtId="2"/>
   </dataFields>
   <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
 </pivotTableDefinition>
@@ -35535,7 +35535,7 @@
     <pageField fld="3" hier="-1"/>
   </pageFields>
   <dataFields count="1">
-    <dataField fld="10" subtotal="average"/>
+    <dataField fld="10" subtotal="average" numFmtId="2"/>
   </dataFields>
   <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
 </pivotTableDefinition>
@@ -37569,7 +37569,7 @@
     <pageField fld="3" hier="-1"/>
   </pageFields>
   <dataFields count="1">
-    <dataField fld="9" subtotal="average"/>
+    <dataField fld="9" subtotal="average" numFmtId="2"/>
   </dataFields>
   <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
 </pivotTableDefinition>
@@ -37736,7 +37736,7 @@
     <pageField fld="3" hier="-1"/>
   </pageFields>
   <dataFields count="1">
-    <dataField fld="9" subtotal="average"/>
+    <dataField fld="9" subtotal="average" numFmtId="2"/>
   </dataFields>
   <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
 </pivotTableDefinition>

</xml_diff>